<commit_message>
Add selective Major Concerns and editable Word wrapping
</commit_message>
<xml_diff>
--- a/skills/minxin-subject-sow-planner/assets/minxin-subject-sow-planner.xlsx
+++ b/skills/minxin-subject-sow-planner/assets/minxin-subject-sow-planner.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="1" r:id="Ree8dcaceedfe4222"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Course_Brief" sheetId="2" r:id="Rda16ce96e4d14084"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendar_Events" sheetId="3" r:id="R46006f0c170147e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timetable_Slots" sheetId="4" r:id="R5670aba4704c4afe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Units" sheetId="5" r:id="Ra94044d8e640463f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Objectives" sheetId="6" r:id="R42be50cd52e54cb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly_Plan" sheetId="7" r:id="Rbf62718c766d448c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weeks" sheetId="8" r:id="R5836ff74584e46f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOW_View" sheetId="9" r:id="R64f23d278ad042b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="10" r:id="R28c629102d094277"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="1" r:id="R0d94b5ddd21b4a74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Course_Brief" sheetId="2" r:id="R2fd0573f07ce4c7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendar_Events" sheetId="3" r:id="Rfbe1e7329a6a4d21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timetable_Slots" sheetId="4" r:id="R9da70398761f47e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Units" sheetId="5" r:id="R69768fc458c5412d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Objectives" sheetId="6" r:id="Rea1af0e2e7d043f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly_Plan" sheetId="7" r:id="R569e4701ff744b22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weeks" sheetId="8" r:id="Ra6ecd19dab7a4fd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOW_View" sheetId="9" r:id="R1e84247e791646bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="10" r:id="Rd05fe3d80a3c4f5f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -448,9 +448,9 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="WeeklyPlanTable" displayName="WeeklyPlanTable" ref="A4:X16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:X16"/>
-  <x:tableColumns count="24">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="WeeklyPlanTable" displayName="WeeklyPlanTable" ref="A4:Y16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:Y16"/>
+  <x:tableColumns count="25">
     <x:tableColumn id="1" name="plan_id"/>
     <x:tableColumn id="2" name="course_id"/>
     <x:tableColumn id="3" name="week_id"/>
@@ -458,23 +458,24 @@
     <x:tableColumn id="5" name="learning_unit"/>
     <x:tableColumn id="6" name="prior_learning"/>
     <x:tableColumn id="7" name="objective_refs"/>
-    <x:tableColumn id="8" name="knowledge_content"/>
-    <x:tableColumn id="9" name="disciplinary_practice"/>
-    <x:tableColumn id="10" name="activities"/>
-    <x:tableColumn id="11" name="evidence"/>
-    <x:tableColumn id="12" name="assessment_purpose"/>
-    <x:tableColumn id="13" name="feedback_revision"/>
-    <x:tableColumn id="14" name="resources"/>
-    <x:tableColumn id="15" name="values"/>
-    <x:tableColumn id="16" name="planned_periods"/>
-    <x:tableColumn id="17" name="available_periods"/>
-    <x:tableColumn id="18" name="repetition_purpose"/>
-    <x:tableColumn id="19" name="progression_delta"/>
-    <x:tableColumn id="20" name="context_delta"/>
-    <x:tableColumn id="21" name="evidence_delta"/>
-    <x:tableColumn id="22" name="independence_delta"/>
-    <x:tableColumn id="23" name="owner"/>
-    <x:tableColumn id="24" name="status"/>
+    <x:tableColumn id="8" name="major_concern_refs"/>
+    <x:tableColumn id="9" name="knowledge_content"/>
+    <x:tableColumn id="10" name="disciplinary_practice"/>
+    <x:tableColumn id="11" name="activities"/>
+    <x:tableColumn id="12" name="evidence"/>
+    <x:tableColumn id="13" name="assessment_purpose"/>
+    <x:tableColumn id="14" name="feedback_revision"/>
+    <x:tableColumn id="15" name="resources"/>
+    <x:tableColumn id="16" name="values"/>
+    <x:tableColumn id="17" name="planned_periods"/>
+    <x:tableColumn id="18" name="available_periods"/>
+    <x:tableColumn id="19" name="repetition_purpose"/>
+    <x:tableColumn id="20" name="progression_delta"/>
+    <x:tableColumn id="21" name="context_delta"/>
+    <x:tableColumn id="22" name="evidence_delta"/>
+    <x:tableColumn id="23" name="independence_delta"/>
+    <x:tableColumn id="24" name="owner"/>
+    <x:tableColumn id="25" name="status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -875,7 +876,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda192cd1bdbe40cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0352d4684a4a4740"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -984,7 +985,9 @@
       <x:c r="I5" s="40" t="str">
         <x:v>page 1</x:v>
       </x:c>
-      <x:c r="J5" s="40" t="str"/>
+      <x:c r="J5" s="40" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A6" s="41" t="str">
@@ -1014,7 +1017,9 @@
       <x:c r="I6" s="41" t="str">
         <x:v>page 1</x:v>
       </x:c>
-      <x:c r="J6" s="41" t="str"/>
+      <x:c r="J6" s="41" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A7" s="41" t="str">
@@ -1044,7 +1049,9 @@
       <x:c r="I7" s="41" t="str">
         <x:v>page 1</x:v>
       </x:c>
-      <x:c r="J7" s="41" t="str"/>
+      <x:c r="J7" s="41" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A8" s="41" t="str">
@@ -1074,7 +1081,9 @@
       <x:c r="I8" s="41" t="str">
         <x:v>page 1</x:v>
       </x:c>
-      <x:c r="J8" s="41" t="str"/>
+      <x:c r="J8" s="41" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A9" s="41" t="str">
@@ -1104,7 +1113,9 @@
       <x:c r="I9" s="41" t="str">
         <x:v>page 1</x:v>
       </x:c>
-      <x:c r="J9" s="41" t="str"/>
+      <x:c r="J9" s="41" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A10" s="41" t="str">
@@ -1134,7 +1145,9 @@
       <x:c r="I10" s="41" t="str">
         <x:v>page 1</x:v>
       </x:c>
-      <x:c r="J10" s="41" t="str"/>
+      <x:c r="J10" s="41" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A11" s="41" t="str">
@@ -1164,7 +1177,9 @@
       <x:c r="I11" s="41" t="str">
         <x:v>page 1</x:v>
       </x:c>
-      <x:c r="J11" s="41" t="str"/>
+      <x:c r="J11" s="41" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A12" s="41" t="str">
@@ -1194,7 +1209,9 @@
       <x:c r="I12" s="41" t="str">
         <x:v>page 1</x:v>
       </x:c>
-      <x:c r="J12" s="41" t="str"/>
+      <x:c r="J12" s="41" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A13" s="41" t="str">
@@ -1224,7 +1241,9 @@
       <x:c r="I13" s="41" t="str">
         <x:v>page 2</x:v>
       </x:c>
-      <x:c r="J13" s="41" t="str"/>
+      <x:c r="J13" s="41" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A14" s="41" t="str">
@@ -1254,7 +1273,9 @@
       <x:c r="I14" s="41" t="str">
         <x:v>page 2</x:v>
       </x:c>
-      <x:c r="J14" s="41" t="str"/>
+      <x:c r="J14" s="41" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A15" s="41" t="str">
@@ -1284,7 +1305,9 @@
       <x:c r="I15" s="41" t="str">
         <x:v>page 2</x:v>
       </x:c>
-      <x:c r="J15" s="41" t="str"/>
+      <x:c r="J15" s="41" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A16" s="41" t="str">
@@ -1314,7 +1337,9 @@
       <x:c r="I16" s="41" t="str">
         <x:v>page 2</x:v>
       </x:c>
-      <x:c r="J16" s="41" t="str"/>
+      <x:c r="J16" s="41" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A17" s="41" t="str">
@@ -1344,7 +1369,9 @@
       <x:c r="I17" s="41" t="str">
         <x:v>page 2</x:v>
       </x:c>
-      <x:c r="J17" s="41" t="str"/>
+      <x:c r="J17" s="41" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A18" s="41" t="str">
@@ -1374,7 +1401,9 @@
       <x:c r="I18" s="41" t="str">
         <x:v>page 2</x:v>
       </x:c>
-      <x:c r="J18" s="41" t="str"/>
+      <x:c r="J18" s="41" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A19" s="41" t="str">
@@ -1404,7 +1433,9 @@
       <x:c r="I19" s="41" t="str">
         <x:v>page 2</x:v>
       </x:c>
-      <x:c r="J19" s="41" t="str"/>
+      <x:c r="J19" s="41" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A20" s="41" t="str">
@@ -1434,7 +1465,9 @@
       <x:c r="I20" s="41" t="str">
         <x:v>page 2</x:v>
       </x:c>
-      <x:c r="J20" s="41" t="str"/>
+      <x:c r="J20" s="41" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A21" s="41" t="str">
@@ -1464,7 +1497,9 @@
       <x:c r="I21" s="41" t="str">
         <x:v>page 2</x:v>
       </x:c>
-      <x:c r="J21" s="41" t="str"/>
+      <x:c r="J21" s="41" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A22" s="41" t="str">
@@ -1494,7 +1529,9 @@
       <x:c r="I22" s="41" t="str">
         <x:v>page 2</x:v>
       </x:c>
-      <x:c r="J22" s="41" t="str"/>
+      <x:c r="J22" s="41" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A23" s="41" t="str">
@@ -1524,7 +1561,9 @@
       <x:c r="I23" s="41" t="str">
         <x:v>page 2</x:v>
       </x:c>
-      <x:c r="J23" s="41" t="str"/>
+      <x:c r="J23" s="41" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A24" s="41" t="str">
@@ -1554,7 +1593,9 @@
       <x:c r="I24" s="41" t="str">
         <x:v>page 2</x:v>
       </x:c>
-      <x:c r="J24" s="41" t="str"/>
+      <x:c r="J24" s="41" t="str">
+        <x:v>Confirm the event scope and policy or record a manual override.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1568,7 +1609,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb365cab3202b4aff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0395f1ca3a884d91"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1842,7 +1883,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5863d4894b23451f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R607afbc885b14dc9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4938,7 +4979,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R622ee17cae9d4f28"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc682f63471f4bb7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5109,7 +5150,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb266b640c85740a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd75a38c19f834b82"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5128,7 +5169,7 @@
     <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="21" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="25" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="13" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="12" hidden="0" customWidth="1"/>
@@ -5154,7 +5195,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>EDITABLE subject units. Major Concerns require observable evidence and normally map at unit level.</x:v>
+        <x:v>EDITABLE subject units. Use Major Concerns here as the broad planning map and require observable evidence.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -5293,7 +5334,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcee64e247b764235"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce2cc87a64334db0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5444,7 +5485,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R555e309a2d824e61"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f2216bf3d0344ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5460,23 +5501,24 @@
     <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="32" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="32" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="42" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="38" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="54" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="42" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="30" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="42" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="34" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="24" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="18" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="20" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="21" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="34" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="42" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="38" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="54" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="42" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="30" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="42" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="34" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="24" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="20" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="21" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="34" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="34" hidden="0" customWidth="1"/>
     <x:col min="22" max="22" width="34" hidden="0" customWidth="1"/>
-    <x:col min="23" max="23" width="12" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="34" hidden="0" customWidth="1"/>
     <x:col min="24" max="24" width="12" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -5506,10 +5548,11 @@
       <x:c r="V1" s="3"/>
       <x:c r="W1" s="3"/>
       <x:c r="X1" s="3"/>
+      <x:c r="Y1" s="3"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>EDITABLE SINGLE SOURCE OF TRUTH. Word and generated views are derived from these rows.</x:v>
+        <x:v>EDITABLE SINGLE SOURCE OF TRUTH. Cite MC1-MC3 only for directly aligned objectives; leave blank otherwise.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -5534,6 +5577,7 @@
       <x:c r="V2" s="6"/>
       <x:c r="W2" s="6"/>
       <x:c r="X2" s="6"/>
+      <x:c r="Y2" s="6"/>
     </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="12" t="str">
@@ -5558,54 +5602,57 @@
         <x:v>objective_refs</x:v>
       </x:c>
       <x:c r="H4" s="12" t="str">
+        <x:v>major_concern_refs</x:v>
+      </x:c>
+      <x:c r="I4" s="12" t="str">
         <x:v>knowledge_content</x:v>
       </x:c>
-      <x:c r="I4" s="12" t="str">
+      <x:c r="J4" s="12" t="str">
         <x:v>disciplinary_practice</x:v>
       </x:c>
-      <x:c r="J4" s="12" t="str">
+      <x:c r="K4" s="12" t="str">
         <x:v>activities</x:v>
       </x:c>
-      <x:c r="K4" s="12" t="str">
+      <x:c r="L4" s="12" t="str">
         <x:v>evidence</x:v>
       </x:c>
-      <x:c r="L4" s="12" t="str">
+      <x:c r="M4" s="12" t="str">
         <x:v>assessment_purpose</x:v>
       </x:c>
-      <x:c r="M4" s="12" t="str">
+      <x:c r="N4" s="12" t="str">
         <x:v>feedback_revision</x:v>
       </x:c>
-      <x:c r="N4" s="12" t="str">
+      <x:c r="O4" s="12" t="str">
         <x:v>resources</x:v>
       </x:c>
-      <x:c r="O4" s="12" t="str">
+      <x:c r="P4" s="12" t="str">
         <x:v>values</x:v>
       </x:c>
-      <x:c r="P4" s="12" t="str">
+      <x:c r="Q4" s="12" t="str">
         <x:v>planned_periods</x:v>
       </x:c>
-      <x:c r="Q4" s="12" t="str">
+      <x:c r="R4" s="12" t="str">
         <x:v>available_periods</x:v>
       </x:c>
-      <x:c r="R4" s="12" t="str">
+      <x:c r="S4" s="12" t="str">
         <x:v>repetition_purpose</x:v>
       </x:c>
-      <x:c r="S4" s="12" t="str">
+      <x:c r="T4" s="12" t="str">
         <x:v>progression_delta</x:v>
       </x:c>
-      <x:c r="T4" s="12" t="str">
+      <x:c r="U4" s="12" t="str">
         <x:v>context_delta</x:v>
       </x:c>
-      <x:c r="U4" s="12" t="str">
+      <x:c r="V4" s="12" t="str">
         <x:v>evidence_delta</x:v>
       </x:c>
-      <x:c r="V4" s="12" t="str">
+      <x:c r="W4" s="12" t="str">
         <x:v>independence_delta</x:v>
       </x:c>
-      <x:c r="W4" s="12" t="str">
+      <x:c r="X4" s="12" t="str">
         <x:v>owner</x:v>
       </x:c>
-      <x:c r="X4" s="12" t="str">
+      <x:c r="Y4" s="12" t="str">
         <x:v>status</x:v>
       </x:c>
     </x:row>
@@ -5634,6 +5681,7 @@
       <x:c r="V5" s="19" t="str"/>
       <x:c r="W5" s="19" t="str"/>
       <x:c r="X5" s="19" t="str"/>
+      <x:c r="Y5" s="19" t="str"/>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="20" t="str"/>
@@ -5660,6 +5708,7 @@
       <x:c r="V6" s="20" t="str"/>
       <x:c r="W6" s="20" t="str"/>
       <x:c r="X6" s="20" t="str"/>
+      <x:c r="Y6" s="20" t="str"/>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="20" t="str"/>
@@ -5686,6 +5735,7 @@
       <x:c r="V7" s="20" t="str"/>
       <x:c r="W7" s="20" t="str"/>
       <x:c r="X7" s="20" t="str"/>
+      <x:c r="Y7" s="20" t="str"/>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="20" t="str"/>
@@ -5712,6 +5762,7 @@
       <x:c r="V8" s="20" t="str"/>
       <x:c r="W8" s="20" t="str"/>
       <x:c r="X8" s="20" t="str"/>
+      <x:c r="Y8" s="20" t="str"/>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="20" t="str"/>
@@ -5738,6 +5789,7 @@
       <x:c r="V9" s="20" t="str"/>
       <x:c r="W9" s="20" t="str"/>
       <x:c r="X9" s="20" t="str"/>
+      <x:c r="Y9" s="20" t="str"/>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="20" t="str"/>
@@ -5764,6 +5816,7 @@
       <x:c r="V10" s="20" t="str"/>
       <x:c r="W10" s="20" t="str"/>
       <x:c r="X10" s="20" t="str"/>
+      <x:c r="Y10" s="20" t="str"/>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="20" t="str"/>
@@ -5790,6 +5843,7 @@
       <x:c r="V11" s="20" t="str"/>
       <x:c r="W11" s="20" t="str"/>
       <x:c r="X11" s="20" t="str"/>
+      <x:c r="Y11" s="20" t="str"/>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="20" t="str"/>
@@ -5816,6 +5870,7 @@
       <x:c r="V12" s="20" t="str"/>
       <x:c r="W12" s="20" t="str"/>
       <x:c r="X12" s="20" t="str"/>
+      <x:c r="Y12" s="20" t="str"/>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="20" t="str"/>
@@ -5842,6 +5897,7 @@
       <x:c r="V13" s="20" t="str"/>
       <x:c r="W13" s="20" t="str"/>
       <x:c r="X13" s="20" t="str"/>
+      <x:c r="Y13" s="20" t="str"/>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="20" t="str"/>
@@ -5868,6 +5924,7 @@
       <x:c r="V14" s="20" t="str"/>
       <x:c r="W14" s="20" t="str"/>
       <x:c r="X14" s="20" t="str"/>
+      <x:c r="Y14" s="20" t="str"/>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="20" t="str"/>
@@ -5894,6 +5951,7 @@
       <x:c r="V15" s="20" t="str"/>
       <x:c r="W15" s="20" t="str"/>
       <x:c r="X15" s="20" t="str"/>
+      <x:c r="Y15" s="20" t="str"/>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="20" t="str"/>
@@ -5920,23 +5978,24 @@
       <x:c r="V16" s="20" t="str"/>
       <x:c r="W16" s="20" t="str"/>
       <x:c r="X16" s="20" t="str"/>
+      <x:c r="Y16" s="20" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:X1"/>
-    <x:mergeCell ref="A2:X2"/>
+    <x:mergeCell ref="A1:Y1"/>
+    <x:mergeCell ref="A2:Y2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="R5:R16">
+    <x:dataValidation type="list" sqref="S5:S16">
       <x:formula1>",RETRIEVAL,CONSOLIDATION,SPIRAL,TRANSFER,ROUTINE"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="X5:X16">
+    <x:dataValidation type="list" sqref="Y5:Y16">
       <x:formula1>"TEST_FIXTURE,PROPOSED_DESIGN,DRAFT,CONFIRMED,CALENDAR_BLOCK"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cb463bc2d934a72"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06a5d7d4e4c64ea5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7408,7 +7467,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd12d67761ca54698"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R451da10cb9314e91"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7429,18 +7488,19 @@
     <x:col min="10" max="10" width="36" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="32" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="32" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="58" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="42" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="38" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="12" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="34" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="24" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="54" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="42" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="30" hidden="0" customWidth="1"/>
-    <x:col min="22" max="22" width="42" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="58" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="42" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="38" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="12" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="34" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="24" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="54" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="42" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="30" hidden="0" customWidth="1"/>
     <x:col min="23" max="23" width="42" hidden="0" customWidth="1"/>
-    <x:col min="24" max="24" width="12" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="42" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -7470,6 +7530,7 @@
       <x:c r="V1" s="3"/>
       <x:c r="W1" s="3"/>
       <x:c r="X1" s="3"/>
+      <x:c r="Y1" s="3"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="34" t="str">
@@ -7498,6 +7559,7 @@
       <x:c r="V2" s="34"/>
       <x:c r="W2" s="34"/>
       <x:c r="X2" s="34"/>
+      <x:c r="Y2" s="34"/>
     </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="12" t="str">
@@ -7537,46 +7599,49 @@
         <x:v>objective_refs</x:v>
       </x:c>
       <x:c r="M4" s="12" t="str">
+        <x:v>major_concern_refs</x:v>
+      </x:c>
+      <x:c r="N4" s="12" t="str">
         <x:v>teaching_objectives</x:v>
       </x:c>
-      <x:c r="N4" s="12" t="str">
+      <x:c r="O4" s="12" t="str">
         <x:v>knowledge_content</x:v>
       </x:c>
-      <x:c r="O4" s="12" t="str">
+      <x:c r="P4" s="12" t="str">
         <x:v>disciplinary_practice</x:v>
       </x:c>
-      <x:c r="P4" s="12" t="str">
+      <x:c r="Q4" s="12" t="str">
         <x:v>periods</x:v>
       </x:c>
-      <x:c r="Q4" s="12" t="str">
+      <x:c r="R4" s="12" t="str">
         <x:v>resources</x:v>
       </x:c>
-      <x:c r="R4" s="12" t="str">
+      <x:c r="S4" s="12" t="str">
         <x:v>values</x:v>
       </x:c>
-      <x:c r="S4" s="12" t="str">
+      <x:c r="T4" s="12" t="str">
         <x:v>activities</x:v>
       </x:c>
-      <x:c r="T4" s="12" t="str">
+      <x:c r="U4" s="12" t="str">
         <x:v>evidence</x:v>
       </x:c>
-      <x:c r="U4" s="12" t="str">
+      <x:c r="V4" s="12" t="str">
         <x:v>assessment_purpose</x:v>
       </x:c>
-      <x:c r="V4" s="12" t="str">
+      <x:c r="W4" s="12" t="str">
         <x:v>feedback_revision</x:v>
       </x:c>
-      <x:c r="W4" s="12" t="str">
+      <x:c r="X4" s="12" t="str">
         <x:v>calendar_context</x:v>
       </x:c>
-      <x:c r="X4" s="12" t="str">
+      <x:c r="Y4" s="12" t="str">
         <x:v>status</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:X1"/>
-    <x:mergeCell ref="A2:X2"/>
+    <x:mergeCell ref="A1:Y1"/>
+    <x:mergeCell ref="A2:Y2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>